<commit_message>
test: add unanswerable QA guardrail rows
</commit_message>
<xml_diff>
--- a/tests/accuracy/StatsChat_QA_Verified_Audited.xlsx
+++ b/tests/accuracy/StatsChat_QA_Verified_Audited.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,7 +522,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="b">
         <v>1</v>
       </c>
@@ -569,7 +568,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="b">
         <v>1</v>
       </c>
@@ -616,7 +614,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="b">
         <v>1</v>
       </c>
@@ -663,7 +660,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="b">
         <v>1</v>
       </c>
@@ -710,7 +706,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="b">
         <v>1</v>
       </c>
@@ -757,7 +752,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="b">
         <v>1</v>
       </c>
@@ -806,7 +800,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="b">
         <v>1</v>
       </c>
@@ -853,7 +846,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="b">
         <v>1</v>
       </c>
@@ -900,7 +892,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="b">
         <v>1</v>
       </c>
@@ -947,7 +938,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="b">
         <v>1</v>
       </c>
@@ -994,7 +984,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="b">
         <v>1</v>
       </c>
@@ -1041,7 +1030,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
         <v>1</v>
       </c>
@@ -1088,7 +1076,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
         <v>1</v>
       </c>
@@ -1137,7 +1124,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="b">
         <v>1</v>
       </c>
@@ -1186,7 +1172,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="b">
         <v>1</v>
       </c>
@@ -1235,7 +1220,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="b">
         <v>1</v>
       </c>
@@ -1284,7 +1268,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="b">
         <v>1</v>
       </c>
@@ -1331,7 +1314,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="b">
         <v>1</v>
       </c>
@@ -1378,7 +1360,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="b">
         <v>1</v>
       </c>
@@ -1425,7 +1406,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="b">
         <v>1</v>
       </c>
@@ -1472,7 +1452,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="b">
         <v>1</v>
       </c>
@@ -1519,7 +1498,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="b">
         <v>1</v>
       </c>
@@ -1566,7 +1544,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="b">
         <v>1</v>
       </c>
@@ -1613,7 +1590,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="b">
         <v>1</v>
       </c>
@@ -1713,7 +1689,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="b">
         <v>1</v>
       </c>
@@ -1760,7 +1735,6 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="b">
         <v>1</v>
       </c>
@@ -1809,7 +1783,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="b">
         <v>1</v>
       </c>
@@ -1856,7 +1829,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="b">
         <v>1</v>
       </c>
@@ -1903,7 +1875,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="b">
         <v>1</v>
       </c>
@@ -1952,7 +1923,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="b">
         <v>1</v>
       </c>
@@ -2001,7 +1971,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="b">
         <v>1</v>
       </c>
@@ -2048,7 +2017,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="b">
         <v>1</v>
       </c>
@@ -2097,7 +2065,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="b">
         <v>1</v>
       </c>
@@ -2146,7 +2113,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="b">
         <v>1</v>
       </c>
@@ -2193,7 +2159,6 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="b">
         <v>1</v>
       </c>
@@ -2242,13 +2207,311 @@
           <t>AA</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="b">
         <v>1</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>Audited against FAISS docstore on 2026-04-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>QQ038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>What was Tanzania's GDP growth rate in 2023?</t>
+        </is>
+      </c>
+      <c r="G39" t="b">
+        <v>0</v>
+      </c>
+      <c r="J39" t="b">
+        <v>1</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Out-of-country; KNBS Kenya corpus only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>QQ039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>How does Uganda's inflation compare to Kenya's in 2024?</t>
+        </is>
+      </c>
+      <c r="G40" t="b">
+        <v>0</v>
+      </c>
+      <c r="J40" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Out-of-country comparison; Uganda data is outside the KNBS Kenya corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>QQ040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>What is the poverty rate in Ethiopia as of 2022?</t>
+        </is>
+      </c>
+      <c r="G41" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Out-of-country; Ethiopia data is outside the KNBS Kenya corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>QQ041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>What was Kenya's inflation rate in December 2026?</t>
+        </is>
+      </c>
+      <c r="G42" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" t="b">
+        <v>1</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Future unavailable data; December 2026 CPI is not published in the corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>QQ042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>What are the results of the 2029 Kenya Census?</t>
+        </is>
+      </c>
+      <c r="G43" t="b">
+        <v>0</v>
+      </c>
+      <c r="J43" t="b">
+        <v>1</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Future unavailable data; 2029 Kenya Census does not exist in the corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>QQ043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Should Kenya reduce interest rates to control inflation?</t>
+        </is>
+      </c>
+      <c r="G44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Policy recommendation; no official statistical answer expected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>QQ044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>What policies should KNBS recommend to reduce poverty in Kenya?</t>
+        </is>
+      </c>
+      <c r="G45" t="b">
+        <v>0</v>
+      </c>
+      <c r="J45" t="b">
+        <v>1</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Policy advice; no official statistical answer expected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>QQ045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Is Kenya's economy performing well compared to its potential?</t>
+        </is>
+      </c>
+      <c r="G46" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" t="b">
+        <v>1</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Subjective judgment; no single official statistical answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>QQ046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Compare Kenya's 2024 CPI inflation with Nigeria's 2024 CPI inflation.</t>
+        </is>
+      </c>
+      <c r="G47" t="b">
+        <v>0</v>
+      </c>
+      <c r="J47" t="b">
+        <v>1</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Cross-country comparison; Nigeria CPI data is outside the KNBS Kenya corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>QQ047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>How does Kenya's KDHS 2022 child mortality compare to Rwanda's DHS?</t>
+        </is>
+      </c>
+      <c r="G48" t="b">
+        <v>0</v>
+      </c>
+      <c r="J48" t="b">
+        <v>1</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Cross-country comparison; Rwanda DHS data is outside the KNBS Kenya corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>QQ048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>What is the salary of the KNBS Director General?</t>
+        </is>
+      </c>
+      <c r="G49" t="b">
+        <v>0</v>
+      </c>
+      <c r="J49" t="b">
+        <v>1</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Personnel/administrative data; not a KNBS statistical publication answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>QQ049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>What is Kenya's military expenditure as a percentage of GDP in 2024?</t>
+        </is>
+      </c>
+      <c r="G50" t="b">
+        <v>0</v>
+      </c>
+      <c r="J50" t="b">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Topic outside indexed KNBS statistical publications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>QQ050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>What is the best county in Kenya?</t>
+        </is>
+      </c>
+      <c r="G51" t="b">
+        <v>0</v>
+      </c>
+      <c r="J51" t="b">
+        <v>1</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Subjective/vague; no single official statistical answer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: add verified answerable QA expansion batch
</commit_message>
<xml_diff>
--- a/tests/accuracy/StatsChat_QA_Verified_Audited.xlsx
+++ b/tests/accuracy/StatsChat_QA_Verified_Audited.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2515,6 +2515,1158 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>QQ051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>What was Kenya's estimated population in 2024?</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>52.4 million</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf p.22</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>"Population (Million) 48.8 49.7 50.6 51.5 52.4"</t>
+        </is>
+      </c>
+      <c r="G52" t="b">
+        <v>1</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J52" t="b">
+        <v>1</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>QQ052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>What was the growth rate of GDP at constant prices in Kenya in 2024?</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>4.7 per cent</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf p.22</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>"Growth of GDP at Constant Prices (Per cent ) (0.3) 7.6 4.9 5.7 4.7"</t>
+        </is>
+      </c>
+      <c r="G53" t="b">
+        <v>1</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J53" t="b">
+        <v>1</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>QQ053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>What was the total wage employment in Kenya's modern sector in 2024?</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>3,213.8 thousand</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf p.38</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>"Public 884.7 923.0 937.8 992.9 1,023.2 Private 1,858.0 1,983.0 2,077.5 2,145.5 2,190.6 Total 2,742.6 2,906.1 3,015.4 3,138.5 3,213.8"</t>
+        </is>
+      </c>
+      <c r="G54" t="b">
+        <v>1</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J54" t="b">
+        <v>1</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>QQ054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>How many people were employed by the Teachers Service Commission in 2024?</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>410.7 thousand</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2025-Facts-and-Figures.pdf p.38</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>"Teachers Service Commission 331.1 349.9 348.6 390.4 410.7"</t>
+        </is>
+      </c>
+      <c r="G55" t="b">
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J55" t="b">
+        <v>1</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>QQ055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>How many holiday and business visitors arrived in Kenya in 2024?</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1,703,361</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2025-Statistical-Abstract.pdf</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2025-Statistical-Abstract.pdf p.280</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>"Holiday/ Business Visitors 1,239,439 1,420,794 1,462,496 1,754,874 1,562,170 305,924 529,937 979,747 1,428,284 1,703,361"</t>
+        </is>
+      </c>
+      <c r="G56" t="b">
+        <v>1</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J56" t="b">
+        <v>1</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>QQ056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>What were Kenya's total visitor arrivals in 2024?</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2,394,376</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2025-Statistical-Abstract.pdf</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2025-Statistical-Abstract.pdf p.281</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>"Total Arrivals 1,459,466 1,666,047 1,778,425 2,027,723 2,035,441 579,560 871,304 1,540,978 2,086,769 2,394,376"</t>
+        </is>
+      </c>
+      <c r="G57" t="b">
+        <v>1</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J57" t="b">
+        <v>1</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>QQ057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>How many tonnes of unmilled wheat did Kenya import in 2024?</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2,313,985.3 tonnes</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2025-Statistical-Abstract.pdf</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2025-Statistical-Abstract.pdf p.190</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>"Wheat, unmilled " 1,362,309.1 1,854,953.8 1,736,691.7 1,998,852.1 1,882,399.8 1,889,921.9 1,676,623.9 2,037,036.0 2,313,985.3"</t>
+        </is>
+      </c>
+      <c r="G58" t="b">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J58" t="b">
+        <v>1</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>QQ058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>How many tonnes of maize were produced in Kenya according to the 2025 Agriculture Production Report?</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>4,028,320 tonnes</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf p.17</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>"In Kenya, maize is the most significant crop, both in terms of cultivated area and total production. It was grown on 2,407,025 hectares and produced 4,028,320 tonnes"</t>
+        </is>
+      </c>
+      <c r="G59" t="b">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J59" t="b">
+        <v>1</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>QQ059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>What was the area under maize cultivation in Kenya in 2024?</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2,407,025 hectares</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf p.17</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>"It was grown on 2,407,025 hectares and produced 4,028,320 tonnes"</t>
+        </is>
+      </c>
+      <c r="G60" t="b">
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J60" t="b">
+        <v>1</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>QQ060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>How many tonnes of Irish potatoes were produced in Kenya according to the 2025 Agriculture Production Report?</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2,149,979 tonnes</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf p.17</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>"Irish potatoes emerged as the second most productive crop, generating 2,149,979 tonnes from 225,976 hectares"</t>
+        </is>
+      </c>
+      <c r="G61" t="b">
+        <v>1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J61" t="b">
+        <v>1</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>QQ061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>What was the construction inflation rate in Kenya in Q4 2024?</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>0.87%</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Construction-Input-Price-Indices-for-Fourth-Quarter-2024.pdf</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Construction-Input-Price-Indices-for-Fourth-Quarter-2024.pdf p.2</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>"The construction inflation rate was 0.87 per cent in Q4-2024"</t>
+        </is>
+      </c>
+      <c r="G62" t="b">
+        <v>1</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J62" t="b">
+        <v>1</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>QQ062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>What share of Kenya's total stock of foreign liabilities came from Europe at the end of 2023?</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>United Kingdom accounted for 46.4 per cent and the Netherlands 17.3 per cent of the total stock from Europe</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2024-Foreign-Investment-Survey-Report.pdf</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2024-Foreign-Investment-Survey-Report.pdf p.8</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>"the United Kingdom and the Netherlands, which accounted for 46.4 per cent and 17.3 per cent, of the total stock of foreign liabilities from Europe, respectively"</t>
+        </is>
+      </c>
+      <c r="G63" t="b">
+        <v>1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J63" t="b">
+        <v>1</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>QQ063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>What percentage of Kenya's total foreign liabilities came from Africa at the end of 2023?</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>26.4 per cent</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2024-Foreign-Investment-Survey-Report.pdf</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2024-Foreign-Investment-Survey-Report.pdf p.8</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>"Africa emerged as the second largest source of foreign liabilities, accounting for 26.4 per cent of the total stock of foreign liabilities at the end of 2023"</t>
+        </is>
+      </c>
+      <c r="G64" t="b">
+        <v>1</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J64" t="b">
+        <v>1</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>QQ064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>What was Kenya's formal financial access rate in 2024?</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>84.8 per cent</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf p.9</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>"Formal financial access increased from 83.7 percent in 2021 to 84.8 percent in 2024"</t>
+        </is>
+      </c>
+      <c r="G65" t="b">
+        <v>1</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J65" t="b">
+        <v>1</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>QQ065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>What percentage of Kenyans used mobile money daily in 2024?</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>52.6 per cent</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf p.10</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>"52.6 percent of Kenyans now use mobile money daily"</t>
+        </is>
+      </c>
+      <c r="G66" t="b">
+        <v>1</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J66" t="b">
+        <v>1</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>QQ066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>What percentage of Kenyans were financially healthy in 2024?</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>18.3 per cent</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf p.11</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>"Financial health remains low, with 18.3 percent of Kenyans financially healthy compared to 17.1 percent in 2021"</t>
+        </is>
+      </c>
+      <c r="G67" t="b">
+        <v>1</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J67" t="b">
+        <v>1</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>QQ067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Which county had the highest working population in Kenya as of 2022?</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Nairobi City, with 2,191,913</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2024-Gross-County-Product.pdf</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2024-Gross-County-Product.pdf p.19</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>"Nairobi City has the highest working population, at 2,191,913"</t>
+        </is>
+      </c>
+      <c r="G68" t="b">
+        <v>1</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J68" t="b">
+        <v>1</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>QQ068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>What was the leading cause of registered health facility deaths in Mombasa County in 2024?</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Pneumonia (424 deaths)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Kenya-Vital-Statistics-Report-2024.pdf</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Kenya-Vital-Statistics-Report-2024.pdf p.212</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>"001: MOMBASA Rank Cause of Death Total 1 Pneumonia 424"</t>
+        </is>
+      </c>
+      <c r="G69" t="b">
+        <v>1</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J69" t="b">
+        <v>1</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>QQ069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>What was the volume of export traffic through the port of Mombasa in 2023?</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>4,950 thousand metric tonnes</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2024-Economic-Survey.pdf</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2024-Economic-Survey.pdf p.327</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>"4,950"; "The volume in metric tonnes of export traffic through the port of Mombasa in 2023, a rise from 4,771 thousand metric tonnes recorded in 2022"</t>
+        </is>
+      </c>
+      <c r="G70" t="b">
+        <v>1</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J70" t="b">
+        <v>1</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>QQ070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>What was Kenya's broad money supply (M3) in August 2023?</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>KSh 5,774,645 million</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Leading-Economic-Indicators-August-2024.pdf</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Leading-Economic-Indicators-August-2024.pdf p.14</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>"August 2,086,516 2,359,553 4,446,069 1,328,576 5,774,645 1.78"</t>
+        </is>
+      </c>
+      <c r="G71" t="b">
+        <v>1</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J71" t="b">
+        <v>1</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>QQ071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>According to the 2024 FinAccess Survey, which livelihood group had the highest formal financial access rate?</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>The employed, at 96.9 per cent</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2024-FinAccess-Household-Survey-Report.pdf p.30</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>"The employed and those who own businesses had the highest access to financial services through formal channels at 96.9 percent and 92.3 percent, respectively"</t>
+        </is>
+      </c>
+      <c r="G72" t="b">
+        <v>1</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J72" t="b">
+        <v>1</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>QQ072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>What were the top three export destinations for Kenyan coffee in the 2023/24 coffee year?</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Belgium (16.8%), USA (16.1%), and Germany (11.4%)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf p.86</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>"the top leading export destinations for Kenyan coffee in the 2023/24 coffee year were Belgium, USA and Germany at 16.8 per cent, 16.1 per cent and 11.4 per cent, respectively"</t>
+        </is>
+      </c>
+      <c r="G73" t="b">
+        <v>1</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J73" t="b">
+        <v>1</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>QQ073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Which county had the largest meat goat population in Kenya in 2024?</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Turkana, with 8,625.2 thousand</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf p.144</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>"Top 10 Meat Goats Rearing Counties, 2024 8,625.2 ... Turkana"</t>
+        </is>
+      </c>
+      <c r="G74" t="b">
+        <v>1</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J74" t="b">
+        <v>1</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>QQ074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>What was the second most widely cultivated crop in Kenya after maize?</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Beans, covering 1,229,611 hectares</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>National-Agriculture-Production-Report-2025.pdf p.17</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>"Beans were the second most widely cultivated crop, covering 1,229,611 hectares and yielding 759,006 tonnes"</t>
+        </is>
+      </c>
+      <c r="G75" t="b">
+        <v>1</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="J75" t="b">
+        <v>1</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(cloud): add report-family routing for expanded QA set
Add report-family cues for Facts & Figures, Statistical Abstract, Construction Input Price Indices, FinAccess, and Leading Economic Indicators so retrieval can route expanded benchmark questions to the right publication families.

Clarify ambiguous audited QA rows and expand QQ031's gold answer with the source percentage. Improve evaluator numeric matching for KNBS ('000) table units and make saved-run rescoring recompute answer correctness while tolerating blank debug fields in reports.

Validated with 67 targeted unit tests and the 2026-04-16_171338 cloud benchmark: answerable accuracy 56/61, unanswerable accuracy 13/13, Pipeline Doc Hit@8 54/61.
</commit_message>
<xml_diff>
--- a/tests/accuracy/StatsChat_QA_Verified_Audited.xlsx
+++ b/tests/accuracy/StatsChat_QA_Verified_Audited.xlsx
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Mobile Phone</t>
+          <t>Mobile phone, 94%</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Audited against FAISS docstore on 2026-04-02.</t>
+          <t>Audited against FAISS docstore on 2026-04-02. Gold answer expanded on 2026-04-16 to include the percentage present in source_text so correct model answers with the value score deterministically.</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>What share of Kenya's total stock of foreign liabilities came from Europe at the end of 2023?</t>
+          <t>Which European countries accounted for the largest shares of Kenya's foreign liabilities from Europe at the end of 2023, and what were their shares?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex. Query clarified on 2026-04-16 to ask for within-Europe country shares, matching the audited gold answer.</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>What was the second most widely cultivated crop in Kenya after maize?</t>
+          <t>What was the second most widely cultivated crop in Kenya after maize, and what area did it cover?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex.</t>
+          <t>Verified against data/json_split indexed chunk on 2026-04-14; drafted by Claude and checked by Codex. Query clarified on 2026-04-16 to ask for the area included in the audited gold answer.</t>
         </is>
       </c>
     </row>

</xml_diff>